<commit_message>
test(session-grants): record comprehensive final verification
Record the fresh comprehensive Docker verification, refresh actual UI/check-in/export artifacts, and retain the review-only mobile-reflow click correction proven by two exact UI-01–14 + REPORT-01–03 Docker E2E passes. No product requirement or assertion changed. No push.
</commit_message>
<xml_diff>
--- a/docs/superpowers/verification/admin-session-grants/review-artifacts/checkins_Session_Grant_Review_Event_A.xlsx
+++ b/docs/superpowers/verification/admin-session-grants/review-artifacts/checkins_Session_Grant_Review_Event_A.xlsx
@@ -475,13 +475,13 @@
         <v>Review Active Session 2</v>
       </c>
       <c r="K2" t="str">
-        <v>30 ก.ย. 2569 22:43:35</v>
+        <v>01 ต.ค. 2569 07:10:39</v>
       </c>
       <c r="L2" t="str">
         <v>Admin Grant</v>
       </c>
       <c r="M2" t="str">
-        <v>30 ก.ย. 2569 22:40:44</v>
+        <v>01 ต.ค. 2569 07:07:39</v>
       </c>
       <c r="N2" t="str">
         <v>Review Admin</v>

</xml_diff>